<commit_message>
Add OpenAPI specification for the dealer API
OpenAPI 3.1 contract: orders, stock, products, invoices, invoice
acknowledgement and health endpoints, two signed webhooks, OAuth2 client
credentials with scopes, RFC 9457 problem details with the error code
catalogue as enumerations, 42 schemas and worked examples. Field mapping
1.1 adds the per-order sequence field to the status event; error
scenario open point E1 is resolved. README marks the specification as
done.
</commit_message>
<xml_diff>
--- a/analysis/04_field_mapping.xlsx
+++ b/analysis/04_field_mapping.xlsx
@@ -147,7 +147,7 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Field mapping and data dictionary, version 1.0</t>
+          <t xml:space="preserve">Field mapping and data dictionary, version 1.1</t>
         </is>
       </c>
     </row>
@@ -159,7 +159,7 @@
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Approved</t>
+          <t xml:space="preserve">Approved; 1.1 adds the sequence field to the order status event (error scenarios open point E1)</t>
         </is>
       </c>
     </row>
@@ -2782,12 +2782,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">orderId</t>
+          <t xml:space="preserve">sequence</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">string</t>
+          <t xml:space="preserve">integer</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -2797,29 +2797,29 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">OPOR.U_VK_OrderId</t>
+          <t xml:space="preserve">Connector log</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ORFICHE.DOCODE</t>
+          <t xml:space="preserve">Connector log</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Increases by one per status change of the order; apply events in this order and ignore an event whose sequence is not higher than the last one applied (added in version 1.1)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">dealerOrderNo</t>
+          <t xml:space="preserve">orderId</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">string(30)</t>
+          <t xml:space="preserve">string</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -2829,29 +2829,29 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lookup key: OPOR.DocNum</t>
+          <t xml:space="preserve">OPOR.U_VK_OrderId</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lookup key: ORFICHE.FICHENO</t>
+          <t xml:space="preserve">ORFICHE.DOCODE</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The connector finds the purchase order with this value</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">previousStatus</t>
+          <t xml:space="preserve">dealerOrderNo</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">enum</t>
+          <t xml:space="preserve">string(30)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -2861,24 +2861,24 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Lookup key: OPOR.DocNum</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Lookup key: ORFICHE.FICHENO</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Section 8.1</t>
+          <t xml:space="preserve">The connector finds the purchase order with this value</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">status</t>
+          <t xml:space="preserve">previousStatus</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -2893,12 +2893,12 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">OPOR.U_VK_Status</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ORFICHE.SPECODE or a defined field</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -2910,7 +2910,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">reasonCode</t>
+          <t xml:space="preserve">status</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -2920,98 +2920,98 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">M</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">OPOR.U_VK_Reason</t>
+          <t xml:space="preserve">OPOR.U_VK_Status</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Defined field</t>
+          <t xml:space="preserve">ORFICHE.SPECODE or a defined field</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Present for PENDING_APPROVAL and REJECTED (section 8.2)</t>
+          <t xml:space="preserve">Section 8.1</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">reasonText</t>
+          <t xml:space="preserve">reasonCode</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">string(500)</t>
+          <t xml:space="preserve">enum</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">O</t>
+          <t xml:space="preserve">C</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">OPOR.Comments (appended)</t>
+          <t xml:space="preserve">OPOR.U_VK_Reason</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ORFICHE.GENEXP2</t>
+          <t xml:space="preserve">Defined field</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Representative's comment, in the Accept-Language of onboarding</t>
+          <t xml:space="preserve">Present for PENDING_APPROVAL and REJECTED (section 8.2)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">decidedBy</t>
+          <t xml:space="preserve">reasonText</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">enum</t>
+          <t xml:space="preserve">string(500)</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">O</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">OPOR.Comments (appended)</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ORFICHE.GENEXP2</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SYSTEM, SALES_REPRESENTATIVE, SALES_MANAGER; present for approval decisions</t>
+          <t xml:space="preserve">Representative's comment, in the Accept-Language of onboarding</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">lines</t>
+          <t xml:space="preserve">decidedBy</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">array</t>
+          <t xml:space="preserve">enum</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -3021,29 +3021,29 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">POR1 rows by lineNo</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ORFLINE rows by LINENO_</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Present for APPROVED, ALLOCATED and REJECTED (section 4.2)</t>
+          <t xml:space="preserve">SYSTEM, SALES_REPRESENTATIVE, SALES_MANAGER; present for approval decisions</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">shipment</t>
+          <t xml:space="preserve">lines</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">object</t>
+          <t xml:space="preserve">array</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -3053,132 +3053,132 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">POR1 rows by lineNo</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ORFLINE rows by LINENO_</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Present for SHIPPED (section 4.3)</t>
+          <t xml:space="preserve">Present for APPROVED, ALLOCATED and REJECTED (section 4.2)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">shipment</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">object</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Present for SHIPPED (section 4.3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">invoice</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">object</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">C</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Present for INVOICED: ettn, invoiceNo; the full invoice event follows separately (section 7)</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">4.2 Lines in the event</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="1" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">API field</t>
         </is>
       </c>
-      <c r="B21" s="1" t="inlineStr">
+      <c r="B22" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Type</t>
         </is>
       </c>
-      <c r="C21" s="1" t="inlineStr">
+      <c r="C22" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">M/C</t>
         </is>
       </c>
-      <c r="D21" s="1" t="inlineStr">
+      <c r="D22" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">SAP Business One (POR1)</t>
         </is>
       </c>
-      <c r="E21" s="1" t="inlineStr">
+      <c r="E22" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Logo (ORFLINE)</t>
         </is>
       </c>
-      <c r="F21" s="1" t="inlineStr">
+      <c r="F22" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">lineNo</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">integer</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">M</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Match on LineNum + 1</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Match on LINENO_</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">sku</t>
+          <t xml:space="preserve">lineNo</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">string(20)</t>
+          <t xml:space="preserve">integer</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -3188,12 +3188,12 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Match on LineNum + 1</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Match on LINENO_</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -3205,17 +3205,17 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">dealerItemCode</t>
+          <t xml:space="preserve">sku</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">string(50)</t>
+          <t xml:space="preserve">string(20)</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">M</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -3230,24 +3230,24 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Echo of the request</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">requestedQuantity</t>
+          <t xml:space="preserve">dealerItemCode</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">decimal(12,3)</t>
+          <t xml:space="preserve">string(50)</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">M</t>
+          <t xml:space="preserve">C</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -3262,14 +3262,14 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">As submitted</t>
+          <t xml:space="preserve">Echo of the request</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">approvedQuantity</t>
+          <t xml:space="preserve">requestedQuantity</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -3284,29 +3284,29 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">POR1.Quantity (updated when reduced)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ORFLINE.AMOUNT (updated when reduced)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">0 when the line is removed by the representative</t>
+          <t xml:space="preserve">As submitted</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">unitCode</t>
+          <t xml:space="preserve">approvedQuantity</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">string(3)</t>
+          <t xml:space="preserve">decimal(12,3)</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -3316,61 +3316,61 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">POR1.Quantity (updated when reduced)</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ORFLINE.AMOUNT (updated when reduced)</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0 when the line is removed by the representative</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">unitPrice</t>
+          <t xml:space="preserve">unitCode</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">decimal(12,2)</t>
+          <t xml:space="preserve">string(3)</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">M</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">POR1.Price</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ORFLINE.PRICE</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Net of VAT, from the dealer's price list; present for APPROVED and ALLOCATED</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">currency</t>
+          <t xml:space="preserve">unitPrice</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">string(3)</t>
+          <t xml:space="preserve">decimal(12,2)</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -3380,29 +3380,29 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">OPOR.DocCur</t>
+          <t xml:space="preserve">POR1.Price</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ORFICHE.TRCURR</t>
+          <t xml:space="preserve">ORFLINE.PRICE</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRY</t>
+          <t xml:space="preserve">Net of VAT, from the dealer's price list; present for APPROVED and ALLOCATED</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vatRate</t>
+          <t xml:space="preserve">currency</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">decimal(5,2)</t>
+          <t xml:space="preserve">string(3)</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -3412,132 +3412,132 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">POR1.VatGroup mapped from the rate</t>
+          <t xml:space="preserve">OPOR.DocCur</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ORFLINE.VAT</t>
+          <t xml:space="preserve">ORFICHE.TRCURR</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Percent, section 8.5</t>
+          <t xml:space="preserve">TRY</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">vatRate</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">decimal(5,2)</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">POR1.VatGroup mapped from the rate</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ORFLINE.VAT</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Percent, section 8.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">lineReasonCode</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">enum</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">C</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">For partial approvals: PARTIAL_STOCK, REMOVED_BY_REPRESENTATIVE</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">4.3 Shipment block</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="1" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">API field</t>
         </is>
       </c>
-      <c r="B34" s="1" t="inlineStr">
+      <c r="B35" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Type</t>
         </is>
       </c>
-      <c r="C34" s="1" t="inlineStr">
+      <c r="C35" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">M/O</t>
         </is>
       </c>
-      <c r="D34" s="1" t="inlineStr">
+      <c r="D35" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">SAP Business One (OPOR)</t>
         </is>
       </c>
-      <c r="E34" s="1" t="inlineStr">
+      <c r="E35" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Logo (ORFICHE)</t>
         </is>
       </c>
-      <c r="F34" s="1" t="inlineStr">
+      <c r="F35" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">shippedAt</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">timestamp</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">M</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">OPOR.U_VK_ShippedAt</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Defined field</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">warehouseCode</t>
+          <t xml:space="preserve">shippedAt</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">string(3)</t>
+          <t xml:space="preserve">timestamp</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -3547,29 +3547,29 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">OPOR.U_VK_ShippedAt</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Defined field</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shipping warehouse</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">deliveryNoteNo</t>
+          <t xml:space="preserve">warehouseCode</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">string(16)</t>
+          <t xml:space="preserve">string(3)</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -3579,56 +3579,56 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">OPOR.U_VK_DeliveryNote</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Defined field</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Shipping warehouse</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">carrier</t>
+          <t xml:space="preserve">deliveryNoteNo</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">string(50)</t>
+          <t xml:space="preserve">string(16)</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">O</t>
+          <t xml:space="preserve">M</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">OPOR.U_VK_DeliveryNote</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Defined field</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Carrier name</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">trackingNo</t>
+          <t xml:space="preserve">carrier</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -3643,47 +3643,79 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">OPOR.TrackNo</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Defined field</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Carrier name</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">trackingNo</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">string(50)</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OPOR.TrackNo</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Defined field</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">packages</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">integer</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">O</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Number of parcels</t>
         </is>

</xml_diff>